<commit_message>
Mise a jour des donnees de reference et des images de test
- data/reference.xlsx : remplace par les donnees reelles preparees pour
  la soutenance (le fichier avait ete renomme par erreur en "Refence
  .xlsx", ce qui aurait empeche l'application de le trouver ; corrige).
- data/Capture d'ecran 2026-07-01 010724.png, data/passport-1-jpeg.webp,
  data/phpCDwGn0.jpg : images de test confirmees et ajoutees au depot
  (retirees du .gitignore).
</commit_message>
<xml_diff>
--- a/data/reference.xlsx
+++ b/data/reference.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="21">
   <si>
     <t>nom</t>
   </si>
@@ -34,85 +34,43 @@
     <t>annee_universitaire</t>
   </si>
   <si>
-    <t>DUPONT</t>
-  </si>
-  <si>
-    <t>Jean</t>
-  </si>
-  <si>
-    <t>15/03/1990</t>
-  </si>
-  <si>
-    <t>ABC123456</t>
+    <t>CHEVALIER</t>
+  </si>
+  <si>
+    <t>Gisèle Audrey</t>
+  </si>
+  <si>
+    <t>T7X62TZ79</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>FRA</t>
+  </si>
+  <si>
+    <t>2024-2025</t>
+  </si>
+  <si>
+    <t>SMITH</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>PP3000000</t>
+  </si>
+  <si>
+    <t>OELIAN</t>
+  </si>
+  <si>
+    <t>YAHAYA MOUSSA</t>
+  </si>
+  <si>
+    <t>Moubarak</t>
   </si>
   <si>
     <t>M</t>
-  </si>
-  <si>
-    <t>FRA</t>
-  </si>
-  <si>
-    <t>2024-2025</t>
-  </si>
-  <si>
-    <t>MARTIN</t>
-  </si>
-  <si>
-    <t>Sophie</t>
-  </si>
-  <si>
-    <t>22/07/1995</t>
-  </si>
-  <si>
-    <t>DEF789012</t>
-  </si>
-  <si>
-    <t>F</t>
-  </si>
-  <si>
-    <t>BERNARD</t>
-  </si>
-  <si>
-    <t>Pierre</t>
-  </si>
-  <si>
-    <t>01/12/1988</t>
-  </si>
-  <si>
-    <t>GHI345678</t>
-  </si>
-  <si>
-    <t>2023-2024</t>
-  </si>
-  <si>
-    <t>PETIT</t>
-  </si>
-  <si>
-    <t>Marie</t>
-  </si>
-  <si>
-    <t>30/06/1992</t>
-  </si>
-  <si>
-    <t>JKL901234</t>
-  </si>
-  <si>
-    <t>MOREAU</t>
-  </si>
-  <si>
-    <t>Lucas</t>
-  </si>
-  <si>
-    <t>10/11/1997</t>
-  </si>
-  <si>
-    <t>MNO567890</t>
-  </si>
-  <si>
-    <t>YAHAYA MOUSSA</t>
-  </si>
-  <si>
-    <t>Moubarak</t>
   </si>
   <si>
     <t>NER</t>
@@ -141,7 +99,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,13 +136,13 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -403,10 +360,11 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="5" width="8.71"/>
+    <col customWidth="1" min="1" max="2" width="8.71"/>
+    <col customWidth="1" min="3" max="3" width="13.29"/>
+    <col customWidth="1" min="4" max="5" width="8.71"/>
     <col customWidth="1" min="6" max="6" width="16.0"/>
     <col customWidth="1" min="7" max="7" width="33.71"/>
-    <col customWidth="1" min="8" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -439,134 +397,68 @@
       <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3">
+        <v>34790.0</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="3">
+        <v>29781.0</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="E3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="3">
+        <v>36718.0</v>
+      </c>
+      <c r="E4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>23</v>
-      </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="4">
-        <v>36718.0</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
+    <row r="18" ht="15.75" customHeight="1"/>
+    <row r="19" ht="15.75" customHeight="1"/>
+    <row r="20" ht="15.75" customHeight="1"/>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
     <row r="23" ht="15.75" customHeight="1"/>
@@ -1544,9 +1436,6 @@
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>